<commit_message>
Ground the dataset in published sources
Real tender spec wording (HAL MAT/P/B-12/263), ~45 live supplier listings and
the industry RFQ checklists replace invented conventions. Adds per-layer GSM
stacks, Ntl/Nlt abbreviations, kg/cm2 strength, inch dimensions against an
mm tender, per-Box unit wording, a bundled sub-component, and a
self-contradictory vendor spec label. Provenance in data/SOURCES.md.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvvUM5YEomPd7JHeb1r99B
</commit_message>
<xml_diff>
--- a/data/generated/shakti_quotation_SPPL-QT-2026-27-0318.xlsx
+++ b/data/generated/shakti_quotation_SPPL-QT-2026-27-0318.xlsx
@@ -1199,7 +1199,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Per Box</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -2359,7 +2359,7 @@
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Per 100 Nos</t>
+          <t>Per 100 Box</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">

</xml_diff>